<commit_message>
only bits left to fix and test are group alloc, rota, patrol boats plus reports
</commit_message>
<xml_diff>
--- a/static/WA_field_list.xlsx
+++ b/static/WA_field_list.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="170" uniqueCount="53">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="175" uniqueCount="55">
   <si>
     <t xml:space="preserve">ALL FIELDS</t>
   </si>
@@ -130,6 +130,9 @@
     <t xml:space="preserve">Sail number</t>
   </si>
   <si>
+    <t xml:space="preserve">Sailor is a club member</t>
+  </si>
+  <si>
     <t xml:space="preserve">Total fee</t>
   </si>
   <si>
@@ -173,6 +176,9 @@
   </si>
   <si>
     <t xml:space="preserve">Volunteer status</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Wants Coached racing</t>
   </si>
   <si>
     <t xml:space="preserve">Wants MG</t>
@@ -385,7 +391,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E49"/>
+  <dimension ref="A1:E51"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="27.45"/>
@@ -718,6 +724,9 @@
       <c r="A27" s="1" t="s">
         <v>30</v>
       </c>
+      <c r="D27" s="1" t="s">
+        <v>30</v>
+      </c>
     </row>
     <row r="28" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="1" t="s">
@@ -808,23 +817,14 @@
       <c r="A33" s="1" t="s">
         <v>36</v>
       </c>
+      <c r="D33" s="1" t="s">
+        <v>36</v>
+      </c>
     </row>
     <row r="34" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="B34" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="C34" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="D34" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="E34" s="1" t="s">
-        <v>37</v>
-      </c>
     </row>
     <row r="35" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="1" t="s">
@@ -864,6 +864,15 @@
       <c r="A37" s="1" t="s">
         <v>40</v>
       </c>
+      <c r="B37" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="C37" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="D37" s="1" t="s">
+        <v>40</v>
+      </c>
       <c r="E37" s="1" t="s">
         <v>40</v>
       </c>
@@ -872,15 +881,6 @@
       <c r="A38" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="B38" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="C38" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="D38" s="1" t="s">
-        <v>41</v>
-      </c>
       <c r="E38" s="1" t="s">
         <v>41</v>
       </c>
@@ -889,6 +889,15 @@
       <c r="A39" s="1" t="s">
         <v>42</v>
       </c>
+      <c r="B39" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="C39" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="D39" s="1" t="s">
+        <v>42</v>
+      </c>
       <c r="E39" s="1" t="s">
         <v>42</v>
       </c>
@@ -897,23 +906,14 @@
       <c r="A40" s="1" t="s">
         <v>43</v>
       </c>
+      <c r="E40" s="1" t="s">
+        <v>43</v>
+      </c>
     </row>
     <row r="41" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="B41" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="C41" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="D41" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="E41" s="1" t="s">
-        <v>44</v>
-      </c>
     </row>
     <row r="42" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="1" t="s">
@@ -936,6 +936,15 @@
       <c r="A43" s="1" t="s">
         <v>46</v>
       </c>
+      <c r="B43" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="C43" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="D43" s="1" t="s">
+        <v>46</v>
+      </c>
       <c r="E43" s="1" t="s">
         <v>46</v>
       </c>
@@ -944,15 +953,6 @@
       <c r="A44" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="B44" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="C44" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="D44" s="1" t="s">
-        <v>47</v>
-      </c>
       <c r="E44" s="1" t="s">
         <v>47</v>
       </c>
@@ -961,6 +961,15 @@
       <c r="A45" s="1" t="s">
         <v>48</v>
       </c>
+      <c r="B45" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="C45" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="D45" s="1" t="s">
+        <v>48</v>
+      </c>
       <c r="E45" s="1" t="s">
         <v>48</v>
       </c>
@@ -969,29 +978,26 @@
       <c r="A46" s="1" t="s">
         <v>49</v>
       </c>
+      <c r="E46" s="1" t="s">
+        <v>49</v>
+      </c>
     </row>
     <row r="47" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="B47" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="C47" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="D47" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="E47" s="1" t="s">
-        <v>50</v>
-      </c>
     </row>
     <row r="48" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="1" t="s">
         <v>51</v>
       </c>
+      <c r="B48" s="1" t="s">
+        <v>51</v>
+      </c>
       <c r="C48" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="D48" s="1" t="s">
         <v>51</v>
       </c>
       <c r="E48" s="1" t="s">
@@ -1001,6 +1007,25 @@
     <row r="49" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="1" t="s">
         <v>52</v>
+      </c>
+      <c r="D49" s="1" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="50" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A50" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="C50" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="E50" s="1" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="51" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A51" s="1" t="s">
+        <v>54</v>
       </c>
     </row>
   </sheetData>

</xml_diff>